<commit_message>
Revisión selectores de logout.
</commit_message>
<xml_diff>
--- a/Output/Ficheros/Mascotas.xlsx
+++ b/Output/Ficheros/Mascotas.xlsx
@@ -46,40 +46,55 @@
     <x:t>Enlace</x:t>
   </x:si>
   <x:si>
-    <x:t>PRETTY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Hembra</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Mestizo Bodeguero</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2 años  y   9 meses</x:t>
+    <x:t>ZALAMERO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Macho</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Burro </x:t>
+  </x:si>
+  <x:si>
+    <x:t>5 años  y   7 meses</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Mediano</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> ZALAMERO es nuestro niño bonito, es tan noble que nos tiene enamorados. Cuando lo recogimos venía tan desnutrido que teníamos que no pudiera sobrevivir.  No deberíamos permitir que ningún animal muriera de hambre, sin embargo, la realidad es que como protectora no podemos hacernos cargo de todos los que nos necesitan.  Aunque a Zalamero ya no le va a faltar quien cuide de él. Desde que siente la barriga llena se le ve contento y con ganas de cariños. Es muy tierno.  Necesitamos madrinas y padrinos que nos ayuden. </x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://arcadenoe.org/ficha-580</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OREJOTAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>5 años  y   9 meses</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> OREJOTAS es el burrito más cariñoso y sociable que hemos conocido. Es tan bueno como bonito.  La subida del precio del grano y el heno ha provocado que algunos dueños hayan tenido que ceder a sus equinos.  Nosotros nos hemos hecho cargo de OREJOTAS porque lo necesitaba pero buscamos padrinos que nos ayuden hasta que encontremos una buena familia que le adopte.  </x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://arcadenoe.org/ficha-573</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MELOCOTÓN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Poni</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9 años  y   11 meses</x:t>
   </x:si>
   <x:si>
     <x:t>Pequeño</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve"> Otra de nuestras pequeñas rescatadas del caso de Chiclana. Se encontraba abandonada junto a una jauría de perros que vivían abandonados en mitad de un pinar. Eran alrededor de 13 perros y poco a poco se han ido rescatando cada uno de ellos.  Pretty tiene tan solo 2 añitos, es una perrita bastante tímida, reservada y muy asustona. Tiene que haber sufrido mucho para que desconfíe tanto de las personas. En el momento en el que le das su espacio, ella comienza a abrirse y a acercarse, pero no le gusta que de primeras la invadan.  </x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://arcadenoe.org/ficha-669</x:t>
-  </x:si>
-  <x:si>
-    <x:t>JENNY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Cruce Pekinés</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1 año  y   11 meses</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve"> Jenny vivía junto a sus cuatro hermanos y su madre de una casa en muy malas condiciones. El día que hicimos el rescate, fuimos consciente de la insalubridad que había en esa casa, ya que vivían entre basura, sus propios excrementos, bichos y suciedad por todos lados.   Es extremadamente miedica, tiene temor a los humanos, aunque con muchísimo trabajo y paciencia, estamos consiguiendo que coma de nuestra mano.   Es una perrita que necesita una estabilidad y una familia que sea capaz de trabajar desde 0, tanto la socialización con los humanos, como el simple hecho de ponerle una correa. No conoce las normas básicas de un hogar, ni controla sus necesidades puesto que no tiene rutinas. Desde que nació ha vivido encerrada sin ningún estímulo.   Si crees que puedes ayudarla, contacta con nosotros. </x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://arcadenoe.org/ficha-653</x:t>
+    <x:t xml:space="preserve"> Nos llegó un aviso de que había entrado un poni en la perrera de Sevilla, aunque nos sorprendió luego aprendimos que por desgracia no es un caso raro. Los equinos también acaban malviviendo en la perrera municipal, y si para los perros es un mal sitio para ellos es aún peor. Nos pusimos manos a la obra y conseguimos sacarlo de allí, ahora vive en nuestro refugio, es muy feliz y nos está enseñando a ser una protectora también de ponis. Es nuestro chico mimado por lo que no se dará en adopción si no es para vivir en mejores condiciones de las que ya está.  Melocontón no es una herramienta de trabajo, no es un muñeco de juguete, es un ser vivo que necesita cariño y capaz de darlo.  Si crees que en tu vida hay hueco para él, no dudes en escribirnos. </x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://arcadenoe.org/ficha-519</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -511,23 +526,43 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="D3" s="0" t="s">
         <x:v>15</x:v>
-      </x:c>
-      <x:c r="D3" s="0" t="s">
-        <x:v>16</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
         <x:v>11</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G3" s="0" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="G3" s="0" t="s">
+    </x:row>
+    <x:row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <x:c r="A4" s="0" t="s">
         <x:v>18</x:v>
       </x:c>
-    </x:row>
-    <x:row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <x:c r="G4" s="2"/>
+      <x:c r="B4" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="D4" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E4" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="F4" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G4" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <x:c r="G5" s="2"/>

</xml_diff>